<commit_message>
feat: visual regression testing of login functionality
</commit_message>
<xml_diff>
--- a/test-data/02_quality-assurance/test-data-credentials.xlsx
+++ b/test-data/02_quality-assurance/test-data-credentials.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Web Test Automation Engineer\test-data\quality-assurance\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Web Test Automation Engineer\test-data\02_quality-assurance\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{EFD1ACA0-20CF-4E01-BD6C-6E8579A81B61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4ACE7947-2FD3-4DB7-A3DE-058322530A9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{6EB67D7B-B7DA-4506-8A70-6F72183A7A24}"/>
+    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{6EB67D7B-B7DA-4506-8A70-6F72183A7A24}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>Id</t>
   </si>
@@ -67,6 +67,9 @@
   </si>
   <si>
     <t>IHateMichaelangelo</t>
+  </si>
+  <si>
+    <t>Id2</t>
   </si>
 </sst>
 </file>
@@ -418,13 +421,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4BCC0DAD-96FD-4D2E-A8AB-811AD34A038C}">
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="25" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -434,8 +437,11 @@
       <c r="C1" t="s">
         <v>2</v>
       </c>
+      <c r="E1" t="s">
+        <v>11</v>
+      </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -446,7 +452,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -457,7 +463,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -468,7 +474,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>

</xml_diff>